<commit_message>
Criado caso de teste 03
</commit_message>
<xml_diff>
--- a/arquivos/Gestão de Testes/Gerenciamento e Monitoramento dos Testes.xlsx
+++ b/arquivos/Gestão de Testes/Gerenciamento e Monitoramento dos Testes.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="58">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -101,15 +101,24 @@
     <t xml:space="preserve">TSL-005</t>
   </si>
   <si>
+    <t xml:space="preserve">[Portal Sawag Labs] – Validar detalhes de informações do produto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Falha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TDBF-438</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TSL-006</t>
+  </si>
+  <si>
     <t xml:space="preserve">[Portal Sawag Labs] –</t>
   </si>
   <si>
     <t xml:space="preserve">Pendente</t>
   </si>
   <si>
-    <t xml:space="preserve">TSL-006</t>
-  </si>
-  <si>
     <t xml:space="preserve">TSL-007</t>
   </si>
   <si>
@@ -180,6 +189,12 @@
   </si>
   <si>
     <t xml:space="preserve">Alta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Imagem do produto não é exibida ao clicar no item</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baixa</t>
   </si>
 </sst>
 </file>
@@ -191,7 +206,7 @@
     <numFmt numFmtId="165" formatCode="d/m/yyyy"/>
     <numFmt numFmtId="166" formatCode="dd/mm/yy"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -227,12 +242,6 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -290,7 +299,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -311,10 +320,6 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -324,10 +329,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -585,20 +586,20 @@
       </c>
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="4" t="s">
         <v>14</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>45193</v>
       </c>
       <c r="G2" s="3"/>
-      <c r="H2" s="6" t="s">
+      <c r="H2" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="6"/>
-      <c r="J2" s="7"/>
-      <c r="K2" s="6"/>
-      <c r="L2" s="7"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="6"/>
+      <c r="K2" s="5"/>
+      <c r="L2" s="6"/>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
@@ -607,22 +608,22 @@
       <c r="B3" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="5" t="s">
+      <c r="C3" s="5"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="4" t="s">
         <v>14</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>45193</v>
       </c>
-      <c r="G3" s="6"/>
-      <c r="H3" s="6" t="s">
+      <c r="G3" s="5"/>
+      <c r="H3" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="I3" s="6"/>
-      <c r="J3" s="6"/>
-      <c r="K3" s="6"/>
-      <c r="L3" s="6"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="5"/>
     </row>
     <row r="4" customFormat="false" ht="24.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
@@ -631,28 +632,28 @@
       <c r="B4" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="5" t="s">
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="4" t="s">
         <v>20</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>45193</v>
       </c>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6" t="s">
+      <c r="G4" s="5"/>
+      <c r="H4" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="I4" s="5" t="s">
         <v>22</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>45193</v>
       </c>
-      <c r="K4" s="6" t="s">
+      <c r="K4" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="L4" s="8" t="n">
+      <c r="L4" s="7" t="n">
         <v>45194</v>
       </c>
     </row>
@@ -660,387 +661,395 @@
       <c r="A5" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="6" t="s">
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="5" t="s">
         <v>14</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>45193</v>
       </c>
-      <c r="G5" s="10"/>
-      <c r="H5" s="10"/>
-      <c r="I5" s="10"/>
-      <c r="J5" s="10"/>
-      <c r="K5" s="10"/>
-      <c r="L5" s="10"/>
+      <c r="G5" s="8"/>
+      <c r="H5" s="8"/>
+      <c r="I5" s="8"/>
+      <c r="J5" s="8"/>
+      <c r="K5" s="8"/>
+      <c r="L5" s="8"/>
     </row>
     <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="10"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="6" t="s">
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="5" t="s">
         <v>27</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>45193</v>
       </c>
-      <c r="G6" s="10"/>
-      <c r="H6" s="10"/>
-      <c r="I6" s="10"/>
-      <c r="J6" s="10"/>
-      <c r="K6" s="10"/>
-      <c r="L6" s="10"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>45193</v>
+      </c>
+      <c r="K6" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="L6" s="8"/>
     </row>
     <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
-      <c r="E7" s="6" t="s">
-        <v>27</v>
+        <v>29</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="5" t="s">
+        <v>31</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>45193</v>
       </c>
-      <c r="G7" s="10"/>
-      <c r="H7" s="10"/>
-      <c r="I7" s="10"/>
-      <c r="J7" s="10"/>
-      <c r="K7" s="10"/>
-      <c r="L7" s="10"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8"/>
     </row>
     <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="6" t="s">
-        <v>27</v>
+        <v>32</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="5" t="s">
+        <v>31</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>45193</v>
       </c>
-      <c r="G8" s="10"/>
-      <c r="H8" s="10"/>
-      <c r="I8" s="10"/>
-      <c r="J8" s="10"/>
-      <c r="K8" s="10"/>
-      <c r="L8" s="10"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
     </row>
     <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="6" t="s">
-        <v>27</v>
+        <v>33</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="5" t="s">
+        <v>31</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>45193</v>
       </c>
-      <c r="G9" s="10"/>
-      <c r="H9" s="10"/>
-      <c r="I9" s="10"/>
-      <c r="J9" s="10"/>
-      <c r="K9" s="10"/>
-      <c r="L9" s="10"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="8"/>
+      <c r="L9" s="8"/>
     </row>
     <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C10" s="10"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="6" t="s">
-        <v>27</v>
+        <v>34</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="5" t="s">
+        <v>31</v>
       </c>
       <c r="F10" s="3" t="n">
         <v>45193</v>
       </c>
-      <c r="G10" s="10"/>
-      <c r="H10" s="10"/>
-      <c r="I10" s="10"/>
-      <c r="J10" s="10"/>
-      <c r="K10" s="10"/>
-      <c r="L10" s="10"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="8"/>
+      <c r="K10" s="8"/>
+      <c r="L10" s="8"/>
     </row>
     <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C11" s="10"/>
-      <c r="D11" s="10"/>
-      <c r="E11" s="6" t="s">
-        <v>27</v>
+        <v>35</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="5" t="s">
+        <v>31</v>
       </c>
       <c r="F11" s="3" t="n">
         <v>45193</v>
       </c>
-      <c r="G11" s="10"/>
-      <c r="H11" s="10"/>
-      <c r="I11" s="10"/>
-      <c r="J11" s="10"/>
-      <c r="K11" s="10"/>
-      <c r="L11" s="10"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="8"/>
+      <c r="K11" s="8"/>
+      <c r="L11" s="8"/>
     </row>
     <row r="12" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="6" t="s">
-        <v>27</v>
+        <v>36</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="5" t="s">
+        <v>31</v>
       </c>
       <c r="F12" s="3" t="n">
         <v>45193</v>
       </c>
-      <c r="G12" s="10"/>
-      <c r="H12" s="10"/>
-      <c r="I12" s="10"/>
-      <c r="J12" s="10"/>
-      <c r="K12" s="10"/>
-      <c r="L12" s="10"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="8"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
+      <c r="K12" s="8"/>
+      <c r="L12" s="8"/>
     </row>
     <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="6" t="s">
-        <v>27</v>
+        <v>37</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="5" t="s">
+        <v>31</v>
       </c>
       <c r="F13" s="3" t="n">
         <v>45193</v>
       </c>
-      <c r="G13" s="10"/>
-      <c r="H13" s="10"/>
-      <c r="I13" s="10"/>
-      <c r="J13" s="10"/>
-      <c r="K13" s="10"/>
-      <c r="L13" s="10"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="8"/>
+      <c r="J13" s="8"/>
+      <c r="K13" s="8"/>
+      <c r="L13" s="8"/>
     </row>
     <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B14" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
-      <c r="E14" s="6" t="s">
-        <v>27</v>
+        <v>38</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C14" s="8"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="5" t="s">
+        <v>31</v>
       </c>
       <c r="F14" s="3" t="n">
         <v>45193</v>
       </c>
-      <c r="G14" s="10"/>
-      <c r="H14" s="10"/>
-      <c r="I14" s="10"/>
-      <c r="J14" s="10"/>
-      <c r="K14" s="10"/>
-      <c r="L14" s="10"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="8"/>
+      <c r="J14" s="8"/>
+      <c r="K14" s="8"/>
+      <c r="L14" s="8"/>
     </row>
     <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B15" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="6" t="s">
-        <v>27</v>
+        <v>39</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C15" s="8"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="5" t="s">
+        <v>31</v>
       </c>
       <c r="F15" s="3" t="n">
         <v>45193</v>
       </c>
-      <c r="G15" s="10"/>
-      <c r="H15" s="10"/>
-      <c r="I15" s="10"/>
-      <c r="J15" s="10"/>
-      <c r="K15" s="10"/>
-      <c r="L15" s="10"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="8"/>
+      <c r="I15" s="8"/>
+      <c r="J15" s="8"/>
+      <c r="K15" s="8"/>
+      <c r="L15" s="8"/>
     </row>
     <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B16" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C16" s="10"/>
-      <c r="D16" s="10"/>
-      <c r="E16" s="6" t="s">
-        <v>27</v>
+        <v>40</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C16" s="8"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="5" t="s">
+        <v>31</v>
       </c>
       <c r="F16" s="3" t="n">
         <v>45193</v>
       </c>
-      <c r="G16" s="10"/>
-      <c r="H16" s="10"/>
-      <c r="I16" s="10"/>
-      <c r="J16" s="10"/>
-      <c r="K16" s="10"/>
-      <c r="L16" s="10"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="8"/>
+      <c r="I16" s="8"/>
+      <c r="J16" s="8"/>
+      <c r="K16" s="8"/>
+      <c r="L16" s="8"/>
     </row>
     <row r="17" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B17" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="6" t="s">
-        <v>27</v>
+        <v>41</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="5" t="s">
+        <v>31</v>
       </c>
       <c r="F17" s="3" t="n">
         <v>45193</v>
       </c>
-      <c r="G17" s="10"/>
-      <c r="H17" s="10"/>
-      <c r="I17" s="10"/>
-      <c r="J17" s="10"/>
-      <c r="K17" s="10"/>
-      <c r="L17" s="10"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8"/>
+      <c r="I17" s="8"/>
+      <c r="J17" s="8"/>
+      <c r="K17" s="8"/>
+      <c r="L17" s="8"/>
     </row>
     <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="B18" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C18" s="10"/>
-      <c r="D18" s="10"/>
-      <c r="E18" s="6" t="s">
-        <v>27</v>
+        <v>42</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C18" s="8"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="5" t="s">
+        <v>31</v>
       </c>
       <c r="F18" s="3" t="n">
         <v>45193</v>
       </c>
-      <c r="G18" s="10"/>
-      <c r="H18" s="10"/>
-      <c r="I18" s="10"/>
-      <c r="J18" s="10"/>
-      <c r="K18" s="10"/>
-      <c r="L18" s="10"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="8"/>
+      <c r="I18" s="8"/>
+      <c r="J18" s="8"/>
+      <c r="K18" s="8"/>
+      <c r="L18" s="8"/>
     </row>
     <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="B19" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C19" s="10"/>
-      <c r="D19" s="10"/>
-      <c r="E19" s="6" t="s">
-        <v>27</v>
+        <v>43</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C19" s="8"/>
+      <c r="D19" s="8"/>
+      <c r="E19" s="5" t="s">
+        <v>31</v>
       </c>
       <c r="F19" s="3" t="n">
         <v>45193</v>
       </c>
-      <c r="G19" s="10"/>
-      <c r="H19" s="10"/>
-      <c r="I19" s="10"/>
-      <c r="J19" s="10"/>
-      <c r="K19" s="10"/>
-      <c r="L19" s="10"/>
+      <c r="G19" s="8"/>
+      <c r="H19" s="8"/>
+      <c r="I19" s="8"/>
+      <c r="J19" s="8"/>
+      <c r="K19" s="8"/>
+      <c r="L19" s="8"/>
     </row>
     <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="B20" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C20" s="10"/>
-      <c r="D20" s="10"/>
-      <c r="E20" s="6" t="s">
-        <v>27</v>
+        <v>44</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C20" s="8"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="5" t="s">
+        <v>31</v>
       </c>
       <c r="F20" s="3" t="n">
         <v>45193</v>
       </c>
-      <c r="G20" s="10"/>
-      <c r="H20" s="10"/>
-      <c r="I20" s="10"/>
-      <c r="J20" s="10"/>
-      <c r="K20" s="10"/>
-      <c r="L20" s="10"/>
+      <c r="G20" s="8"/>
+      <c r="H20" s="8"/>
+      <c r="I20" s="8"/>
+      <c r="J20" s="8"/>
+      <c r="K20" s="8"/>
+      <c r="L20" s="8"/>
     </row>
     <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="B21" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C21" s="10"/>
-      <c r="D21" s="10"/>
-      <c r="E21" s="6" t="s">
-        <v>27</v>
+        <v>45</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C21" s="8"/>
+      <c r="D21" s="8"/>
+      <c r="E21" s="5" t="s">
+        <v>31</v>
       </c>
       <c r="F21" s="3" t="n">
         <v>45193</v>
       </c>
-      <c r="G21" s="10"/>
-      <c r="H21" s="10"/>
-      <c r="I21" s="10"/>
-      <c r="J21" s="10"/>
-      <c r="K21" s="10"/>
-      <c r="L21" s="10"/>
+      <c r="G21" s="8"/>
+      <c r="H21" s="8"/>
+      <c r="I21" s="8"/>
+      <c r="J21" s="8"/>
+      <c r="K21" s="8"/>
+      <c r="L21" s="8"/>
     </row>
     <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E26" s="11"/>
+      <c r="E26" s="9"/>
     </row>
     <row r="27" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E27" s="11"/>
+      <c r="E27" s="9"/>
     </row>
     <row r="28" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E28" s="11"/>
+      <c r="E28" s="9"/>
     </row>
     <row r="29" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E29" s="12"/>
+      <c r="E29" s="10"/>
     </row>
     <row r="1048535" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048536" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -1119,7 +1128,7 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="21.35"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="20.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="44.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="45.82"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20.95"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="15.13"/>
@@ -1133,25 +1142,25 @@
         <v>9</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="I1" s="2" t="s">
         <v>10</v>
@@ -1161,37 +1170,63 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="25.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="7" t="n">
-        <v>45193</v>
-      </c>
-      <c r="B2" s="6" t="s">
+      <c r="A2" s="6" t="n">
+        <v>45193</v>
+      </c>
+      <c r="B2" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
+      <c r="C2" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
       <c r="F2" s="3" t="s">
         <v>18</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="H2" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="I2" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="I2" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="J2" s="7" t="n">
+      <c r="J2" s="6" t="n">
         <v>45194</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E14" s="3"/>
-      <c r="F14" s="5"/>
-    </row>
+    <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="6" t="n">
+        <v>45193</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J3" s="8"/>
+    </row>
+    <row r="1048563" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048564" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048565" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048566" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -1203,17 +1238,21 @@
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <dataValidations count="3">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2" type="list">
-      <formula1>"Bloqueado,Alta,Média,Baixa"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
+  <dataValidations count="4">
     <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G2" type="list">
       <formula1>"Implementação,Arquitetura,Requisitos"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="I2" type="list">
-      <formula1>"Sim,Não"</formula1>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G3:G11" type="list">
+      <formula1>"Implementação,Arquitetura,Requisitos"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:H12" type="list">
+      <formula1>"Bloqueado,Alta,Média,Baixa"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="I2:I7" type="list">
+      <formula1>"--,Sim,Não"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Atualizado planilha de gestao de testes
</commit_message>
<xml_diff>
--- a/arquivos/Gestão de Testes/Gerenciamento e Monitoramento dos Testes.xlsx
+++ b/arquivos/Gestão de Testes/Gerenciamento e Monitoramento dos Testes.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="67">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -65,6 +65,9 @@
     <t xml:space="preserve">[Portal Sawag Labs] – Realizar login com sucesso</t>
   </si>
   <si>
+    <t xml:space="preserve">Dado que efetuei a autenticacao de usuario com "&lt;username&gt;" e "&lt;password&gt;"     Entao devo visualizar a tela inicial do Swag Labs</t>
+  </si>
+  <si>
     <t xml:space="preserve">Concluído</t>
   </si>
   <si>
@@ -77,6 +80,9 @@
     <t xml:space="preserve">[Portal Sawag Labs] – Realizar compra de um produto com sucesso</t>
   </si>
   <si>
+    <t xml:space="preserve">Dado que efetuei a autenticacao de usuario com sucesso     E realizei a compra de um produto     Entao devo finalizar o pagamento</t>
+  </si>
+  <si>
     <t xml:space="preserve">TSL-003</t>
   </si>
   <si>
@@ -98,12 +104,18 @@
     <t xml:space="preserve">[Portal Sawag Labs] – Remover produto do carrinho de compras</t>
   </si>
   <si>
+    <t xml:space="preserve">Dado que efetuei a autenticacao de usuario com sucesso     E realizei o pedido de um produto     E removi um produto do carrinho de compras     Entao nao devo visualizar o produto no carrinho de compras</t>
+  </si>
+  <si>
     <t xml:space="preserve">TSL-005</t>
   </si>
   <si>
     <t xml:space="preserve">[Portal Sawag Labs] – Validar detalhes de informações do produto</t>
   </si>
   <si>
+    <t xml:space="preserve">Dado que efetuei a autenticacao de usuario com sucesso     E cliquei num produto para ver as informações detalhadas     Entao devo visualizar informações com imagem, nome e descrição do produto</t>
+  </si>
+  <si>
     <t xml:space="preserve">Falha</t>
   </si>
   <si>
@@ -113,21 +125,39 @@
     <t xml:space="preserve">TSL-006</t>
   </si>
   <si>
+    <t xml:space="preserve">[Portal Sawag Labs] – Validar opções no Menu Hamburguer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dado que efetuei a autenticacao de usuario com sucesso     E cliquei no menu hamburguer     Entao devo visualizar os items</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TSL-007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[Portal Sawag Labs] – Realizar autenticação com senha incorreta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dado que efetuei a autenticacao com "&lt;username&gt;" e senha "&lt;password&gt;"     Entao devo visualizar uma mensagem de erro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TSL-008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[Portal Sawag Labs] – Realizar autenticação com username incorreto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dado que efetuei a autenticacao com "&lt;username&gt;" incorreto e "&lt;password&gt;"     Entao devo visualizar uma mensagem de erro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TSL-009</t>
+  </si>
+  <si>
     <t xml:space="preserve">[Portal Sawag Labs] –</t>
   </si>
   <si>
     <t xml:space="preserve">Pendente</t>
   </si>
   <si>
-    <t xml:space="preserve">TSL-007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TSL-008</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TSL-009</t>
-  </si>
-  <si>
     <t xml:space="preserve">TSL-010</t>
   </si>
   <si>
@@ -165,9 +195,6 @@
   </si>
   <si>
     <t xml:space="preserve">Titulo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Descrição do Defeito</t>
   </si>
   <si>
     <t xml:space="preserve">Passo a passo até a Falha/Defeito/Erro</t>
@@ -532,7 +559,7 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="58.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="18.81"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="39.08"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20.27"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="14.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="7" style="1" width="11.53"/>
@@ -577,467 +604,467 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="35.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
         <v>12</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="4"/>
+      <c r="C2" s="4" t="s">
+        <v>14</v>
+      </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>45193</v>
       </c>
       <c r="G2" s="3"/>
       <c r="H2" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I2" s="5"/>
       <c r="J2" s="6"/>
       <c r="K2" s="5"/>
       <c r="L2" s="6"/>
     </row>
-    <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="35.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C3" s="5"/>
+        <v>18</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D3" s="5"/>
       <c r="E3" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>45193</v>
       </c>
       <c r="G3" s="5"/>
       <c r="H3" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I3" s="5"/>
       <c r="J3" s="5"/>
       <c r="K3" s="5"/>
       <c r="L3" s="5"/>
     </row>
-    <row r="4" customFormat="false" ht="24.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="35.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="5"/>
       <c r="D4" s="5"/>
       <c r="E4" s="4" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>45193</v>
       </c>
       <c r="G4" s="5"/>
       <c r="H4" s="5" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>45193</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="L4" s="7" t="n">
         <v>45194</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="58" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
+        <v>26</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" s="5"/>
       <c r="E5" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>45193</v>
       </c>
-      <c r="G5" s="8"/>
-      <c r="H5" s="8"/>
-      <c r="I5" s="8"/>
-      <c r="J5" s="8"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I5" s="5"/>
+      <c r="J5" s="5"/>
       <c r="K5" s="8"/>
-      <c r="L5" s="8"/>
-    </row>
-    <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="L5" s="5"/>
+    </row>
+    <row r="6" customFormat="false" ht="58" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
+        <v>29</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D6" s="5"/>
       <c r="E6" s="5" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>45193</v>
       </c>
-      <c r="G6" s="8"/>
-      <c r="H6" s="8" t="s">
-        <v>21</v>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5" t="s">
+        <v>23</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>45193</v>
       </c>
       <c r="K6" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="L6" s="5"/>
+    </row>
+    <row r="7" customFormat="false" ht="35.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5" t="s">
         <v>15</v>
-      </c>
-      <c r="L6" s="8"/>
-    </row>
-    <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="5" t="s">
-        <v>31</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>45193</v>
       </c>
-      <c r="G7" s="8"/>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I7" s="5"/>
+      <c r="J7" s="5"/>
       <c r="K7" s="8"/>
-      <c r="L7" s="8"/>
-    </row>
-    <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="L7" s="5"/>
+    </row>
+    <row r="8" customFormat="false" ht="35.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
+        <v>37</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D8" s="5"/>
       <c r="E8" s="5" t="s">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>45193</v>
       </c>
-      <c r="G8" s="8"/>
-      <c r="H8" s="8"/>
-      <c r="I8" s="8"/>
-      <c r="J8" s="8"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I8" s="5"/>
+      <c r="J8" s="5"/>
       <c r="K8" s="8"/>
-      <c r="L8" s="8"/>
-    </row>
-    <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="L8" s="5"/>
+    </row>
+    <row r="9" customFormat="false" ht="114.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
+        <v>40</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="D9" s="5"/>
       <c r="E9" s="5" t="s">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>45193</v>
       </c>
-      <c r="G9" s="8"/>
-      <c r="H9" s="8"/>
-      <c r="I9" s="8"/>
-      <c r="J9" s="8"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I9" s="5"/>
+      <c r="J9" s="5"/>
       <c r="K9" s="8"/>
-      <c r="L9" s="8"/>
+      <c r="L9" s="5"/>
     </row>
     <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
+        <v>43</v>
+      </c>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
       <c r="E10" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="F10" s="3" t="n">
-        <v>45193</v>
-      </c>
-      <c r="G10" s="8"/>
-      <c r="H10" s="8"/>
-      <c r="I10" s="8"/>
-      <c r="J10" s="8"/>
+        <v>44</v>
+      </c>
+      <c r="F10" s="3"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5"/>
+      <c r="J10" s="5"/>
       <c r="K10" s="8"/>
-      <c r="L10" s="8"/>
+      <c r="L10" s="5"/>
     </row>
     <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8"/>
+        <v>43</v>
+      </c>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
       <c r="E11" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="F11" s="3" t="n">
-        <v>45193</v>
-      </c>
-      <c r="G11" s="8"/>
-      <c r="H11" s="8"/>
-      <c r="I11" s="8"/>
-      <c r="J11" s="8"/>
+        <v>44</v>
+      </c>
+      <c r="F11" s="3"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="5"/>
+      <c r="I11" s="5"/>
+      <c r="J11" s="5"/>
       <c r="K11" s="8"/>
-      <c r="L11" s="8"/>
+      <c r="L11" s="5"/>
     </row>
     <row r="12" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8"/>
+        <v>43</v>
+      </c>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
       <c r="E12" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="F12" s="3" t="n">
-        <v>45193</v>
-      </c>
-      <c r="G12" s="8"/>
-      <c r="H12" s="8"/>
-      <c r="I12" s="8"/>
-      <c r="J12" s="8"/>
+        <v>44</v>
+      </c>
+      <c r="F12" s="3"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="5"/>
+      <c r="I12" s="5"/>
+      <c r="J12" s="5"/>
       <c r="K12" s="8"/>
-      <c r="L12" s="8"/>
+      <c r="L12" s="5"/>
     </row>
     <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
+        <v>43</v>
+      </c>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
       <c r="E13" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="F13" s="3" t="n">
-        <v>45193</v>
-      </c>
-      <c r="G13" s="8"/>
-      <c r="H13" s="8"/>
-      <c r="I13" s="8"/>
-      <c r="J13" s="8"/>
+        <v>44</v>
+      </c>
+      <c r="F13" s="3"/>
+      <c r="G13" s="5"/>
+      <c r="H13" s="5"/>
+      <c r="I13" s="5"/>
+      <c r="J13" s="5"/>
       <c r="K13" s="8"/>
-      <c r="L13" s="8"/>
+      <c r="L13" s="5"/>
     </row>
     <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C14" s="8"/>
-      <c r="D14" s="8"/>
+        <v>43</v>
+      </c>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
       <c r="E14" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="F14" s="3" t="n">
-        <v>45193</v>
-      </c>
-      <c r="G14" s="8"/>
-      <c r="H14" s="8"/>
-      <c r="I14" s="8"/>
-      <c r="J14" s="8"/>
+        <v>44</v>
+      </c>
+      <c r="F14" s="3"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="5"/>
+      <c r="I14" s="5"/>
+      <c r="J14" s="5"/>
       <c r="K14" s="8"/>
-      <c r="L14" s="8"/>
+      <c r="L14" s="5"/>
     </row>
     <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C15" s="8"/>
-      <c r="D15" s="8"/>
+        <v>43</v>
+      </c>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
       <c r="E15" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="F15" s="3" t="n">
-        <v>45193</v>
-      </c>
-      <c r="G15" s="8"/>
-      <c r="H15" s="8"/>
-      <c r="I15" s="8"/>
-      <c r="J15" s="8"/>
+        <v>44</v>
+      </c>
+      <c r="F15" s="3"/>
+      <c r="G15" s="5"/>
+      <c r="H15" s="5"/>
+      <c r="I15" s="5"/>
+      <c r="J15" s="5"/>
       <c r="K15" s="8"/>
-      <c r="L15" s="8"/>
+      <c r="L15" s="5"/>
     </row>
     <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C16" s="8"/>
-      <c r="D16" s="8"/>
+        <v>43</v>
+      </c>
+      <c r="C16" s="5"/>
+      <c r="D16" s="5"/>
       <c r="E16" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="F16" s="3" t="n">
-        <v>45193</v>
-      </c>
-      <c r="G16" s="8"/>
-      <c r="H16" s="8"/>
-      <c r="I16" s="8"/>
-      <c r="J16" s="8"/>
+        <v>44</v>
+      </c>
+      <c r="F16" s="3"/>
+      <c r="G16" s="5"/>
+      <c r="H16" s="5"/>
+      <c r="I16" s="5"/>
+      <c r="J16" s="5"/>
       <c r="K16" s="8"/>
-      <c r="L16" s="8"/>
+      <c r="L16" s="5"/>
     </row>
     <row r="17" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
+        <v>43</v>
+      </c>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
       <c r="E17" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="F17" s="3" t="n">
-        <v>45193</v>
-      </c>
-      <c r="G17" s="8"/>
-      <c r="H17" s="8"/>
-      <c r="I17" s="8"/>
-      <c r="J17" s="8"/>
+        <v>44</v>
+      </c>
+      <c r="F17" s="3"/>
+      <c r="G17" s="5"/>
+      <c r="H17" s="5"/>
+      <c r="I17" s="5"/>
+      <c r="J17" s="5"/>
       <c r="K17" s="8"/>
-      <c r="L17" s="8"/>
+      <c r="L17" s="5"/>
     </row>
     <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C18" s="8"/>
-      <c r="D18" s="8"/>
+        <v>43</v>
+      </c>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
       <c r="E18" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="F18" s="3" t="n">
-        <v>45193</v>
-      </c>
-      <c r="G18" s="8"/>
-      <c r="H18" s="8"/>
-      <c r="I18" s="8"/>
-      <c r="J18" s="8"/>
+        <v>44</v>
+      </c>
+      <c r="F18" s="3"/>
+      <c r="G18" s="5"/>
+      <c r="H18" s="5"/>
+      <c r="I18" s="5"/>
+      <c r="J18" s="5"/>
       <c r="K18" s="8"/>
-      <c r="L18" s="8"/>
+      <c r="L18" s="5"/>
     </row>
     <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B19" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="B19" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C19" s="8"/>
-      <c r="D19" s="8"/>
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
       <c r="E19" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="F19" s="3" t="n">
-        <v>45193</v>
-      </c>
-      <c r="G19" s="8"/>
-      <c r="H19" s="8"/>
-      <c r="I19" s="8"/>
-      <c r="J19" s="8"/>
+        <v>44</v>
+      </c>
+      <c r="F19" s="3"/>
+      <c r="G19" s="5"/>
+      <c r="H19" s="5"/>
+      <c r="I19" s="5"/>
+      <c r="J19" s="5"/>
       <c r="K19" s="8"/>
-      <c r="L19" s="8"/>
+      <c r="L19" s="5"/>
     </row>
     <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C20" s="5"/>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="B20" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C20" s="8"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="F20" s="3" t="n">
-        <v>45193</v>
-      </c>
-      <c r="G20" s="8"/>
-      <c r="H20" s="8"/>
-      <c r="I20" s="8"/>
-      <c r="J20" s="8"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="5"/>
+      <c r="H20" s="5"/>
+      <c r="I20" s="5"/>
+      <c r="J20" s="5"/>
       <c r="K20" s="8"/>
-      <c r="L20" s="8"/>
+      <c r="L20" s="5"/>
     </row>
     <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C21" s="8"/>
-      <c r="D21" s="8"/>
+        <v>43</v>
+      </c>
+      <c r="C21" s="5"/>
+      <c r="D21" s="5"/>
       <c r="E21" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="F21" s="3" t="n">
-        <v>45193</v>
-      </c>
-      <c r="G21" s="8"/>
-      <c r="H21" s="8"/>
-      <c r="I21" s="8"/>
-      <c r="J21" s="8"/>
+        <v>44</v>
+      </c>
+      <c r="F21" s="3"/>
+      <c r="G21" s="5"/>
+      <c r="H21" s="5"/>
+      <c r="I21" s="5"/>
+      <c r="J21" s="5"/>
       <c r="K21" s="8"/>
-      <c r="L21" s="8"/>
+      <c r="L21" s="5"/>
     </row>
     <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E26" s="9"/>
@@ -1123,77 +1150,73 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J1048576"/>
+  <dimension ref="A1:I1048576"/>
   <sheetFormatPr defaultColWidth="12.01171875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="21.35"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="20.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="45.82"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20.95"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="15.13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="1" width="15.15"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="11.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="16.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="15.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="15.15"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="11.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="16.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="11.53"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="46.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>52</v>
+        <v>10</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J1" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="25.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="n">
         <v>45193</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
+      <c r="E2" s="3" t="s">
+        <v>20</v>
+      </c>
       <c r="F2" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="I2" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="J2" s="6" t="n">
+        <v>63</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I2" s="6" t="n">
         <v>45194</v>
       </c>
     </row>
@@ -1202,26 +1225,25 @@
         <v>45193</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D3" s="5"/>
+      <c r="E3" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="3" t="s">
-        <v>25</v>
+      <c r="F3" s="5" t="s">
+        <v>63</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="J3" s="8"/>
+        <v>16</v>
+      </c>
+      <c r="I3" s="5"/>
     </row>
     <row r="1048563" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048564" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -1239,19 +1261,19 @@
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <dataValidations count="4">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G2" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F2" type="list">
       <formula1>"Implementação,Arquitetura,Requisitos"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G3:G11" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F3:F11" type="list">
       <formula1>"Implementação,Arquitetura,Requisitos"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:H12" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G2:G12" type="list">
       <formula1>"Bloqueado,Alta,Média,Baixa"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="I2:I7" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:H7" type="list">
       <formula1>"--,Sim,Não"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Atualizado arquivos de gestao de testes
</commit_message>
<xml_diff>
--- a/arquivos/Gestão de Testes/Gerenciamento e Monitoramento dos Testes.xlsx
+++ b/arquivos/Gestão de Testes/Gerenciamento e Monitoramento dos Testes.xlsx
@@ -326,7 +326,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -369,6 +369,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1161,7 +1165,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="15.15"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="11.99"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="16.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="11" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Atualizado planilha de gerenciamento
</commit_message>
<xml_diff>
--- a/arquivos/Gestão de Testes/Gerenciamento e Monitoramento dos Testes.xlsx
+++ b/arquivos/Gestão de Testes/Gerenciamento e Monitoramento dos Testes.xlsx
@@ -62,7 +62,7 @@
     <t xml:space="preserve">TSL-001</t>
   </si>
   <si>
-    <t xml:space="preserve">[Portal Sawag Labs] – Realizar login com sucesso</t>
+    <t xml:space="preserve">[Portal Swag Labs] – Realizar login com sucesso</t>
   </si>
   <si>
     <t xml:space="preserve">Dado que efetuei a autenticacao de usuario com "&lt;username&gt;" e "&lt;password&gt;"     Entao devo visualizar a tela inicial do Swag Labs</t>
@@ -77,7 +77,7 @@
     <t xml:space="preserve">TSL-002</t>
   </si>
   <si>
-    <t xml:space="preserve">[Portal Sawag Labs] – Realizar compra de um produto com sucesso</t>
+    <t xml:space="preserve">[Portal Swag Labs] – Realizar compra de um produto com sucesso</t>
   </si>
   <si>
     <t xml:space="preserve">Dado que efetuei a autenticacao de usuario com sucesso     E realizei a compra de um produto     Entao devo finalizar o pagamento</t>
@@ -86,7 +86,7 @@
     <t xml:space="preserve">TSL-003</t>
   </si>
   <si>
-    <t xml:space="preserve">[Portal Sawag Labs] – Validar detalhes de pagamento antes de finalizar compra</t>
+    <t xml:space="preserve">[Portal Swag Labs] – Validar detalhes de pagamento antes de finalizar compra</t>
   </si>
   <si>
     <t xml:space="preserve">Bloqueado</t>
@@ -101,7 +101,7 @@
     <t xml:space="preserve">TSL-004</t>
   </si>
   <si>
-    <t xml:space="preserve">[Portal Sawag Labs] – Remover produto do carrinho de compras</t>
+    <t xml:space="preserve">[Portal Swag Labs] – Remover produto do carrinho de compras</t>
   </si>
   <si>
     <t xml:space="preserve">Dado que efetuei a autenticacao de usuario com sucesso     E realizei o pedido de um produto     E removi um produto do carrinho de compras     Entao nao devo visualizar o produto no carrinho de compras</t>
@@ -110,7 +110,7 @@
     <t xml:space="preserve">TSL-005</t>
   </si>
   <si>
-    <t xml:space="preserve">[Portal Sawag Labs] – Validar detalhes de informações do produto</t>
+    <t xml:space="preserve">[Portal Swag Labs] – Validar detalhes de informações do produto</t>
   </si>
   <si>
     <t xml:space="preserve">Dado que efetuei a autenticacao de usuario com sucesso     E cliquei num produto para ver as informações detalhadas     Entao devo visualizar informações com imagem, nome e descrição do produto</t>
@@ -125,7 +125,7 @@
     <t xml:space="preserve">TSL-006</t>
   </si>
   <si>
-    <t xml:space="preserve">[Portal Sawag Labs] – Validar opções no Menu Hamburguer</t>
+    <t xml:space="preserve">[Portal Swag Labs] – Validar opções no Menu Hamburguer</t>
   </si>
   <si>
     <t xml:space="preserve">Dado que efetuei a autenticacao de usuario com sucesso     E cliquei no menu hamburguer     Entao devo visualizar os items</t>
@@ -134,7 +134,7 @@
     <t xml:space="preserve">TSL-007</t>
   </si>
   <si>
-    <t xml:space="preserve">[Portal Sawag Labs] – Realizar autenticação com senha incorreta</t>
+    <t xml:space="preserve">[Portal Swag Labs] – Realizar autenticação com senha incorreta</t>
   </si>
   <si>
     <t xml:space="preserve">Dado que efetuei a autenticacao com "&lt;username&gt;" e senha "&lt;password&gt;"     Entao devo visualizar uma mensagem de erro</t>
@@ -143,7 +143,7 @@
     <t xml:space="preserve">TSL-008</t>
   </si>
   <si>
-    <t xml:space="preserve">[Portal Sawag Labs] – Realizar autenticação com username incorreto</t>
+    <t xml:space="preserve">[Portal Swag Labs] – Realizar autenticação com username incorreto</t>
   </si>
   <si>
     <t xml:space="preserve">Dado que efetuei a autenticacao com "&lt;username&gt;" incorreto e "&lt;password&gt;"     Entao devo visualizar uma mensagem de erro</t>
@@ -152,7 +152,7 @@
     <t xml:space="preserve">TSL-009</t>
   </si>
   <si>
-    <t xml:space="preserve">[Portal Sawag Labs] –</t>
+    <t xml:space="preserve">[Portal Swag Labs] –</t>
   </si>
   <si>
     <t xml:space="preserve">Pendente</t>

</xml_diff>